<commit_message>
feat(schema): model CSF 2.0's functions, categories, subcategories and examples
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/nist_csf_v2.xlsx
+++ b/project/excel/nist_csf_v2.xlsx
@@ -7,22 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CSFDocument" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CSFCatalogBody" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CSFMetadata" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CSFFunction" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CSFCategory" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CSFSubcategory" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CSFPart" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CSFProperty" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Link" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Role" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Party" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Address" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ResponsibleParty" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="BackMatter" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Resource" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ResourceLink" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CsfFramework" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CsfFunction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CsfCategory" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CsfSubcategory" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CsfImplementationExample" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,225 +417,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>catalog</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>csf_version</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>title</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>short-name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>email-addresses</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>addresses</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>addr-lines</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>postal-code</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>role-id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>party-uuids</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resources</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>rlinks</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>href</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>media-type</t>
+          <t>functions</t>
         </is>
       </c>
     </row>
@@ -667,22 +449,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>uuid</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>groups</t>
+          <t>function_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>back-matter</t>
+          <t>function_categories</t>
         </is>
       </c>
     </row>
@@ -697,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -708,51 +490,41 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>published</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>last-modified</t>
+          <t>category_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>category_subcategories</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>oscal-version</t>
+          <t>category_status</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>props</t>
+          <t>category_moved_to</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>links</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>roles</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>parties</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>responsible-parties</t>
+          <t>category_incorporated_into</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"withdrawn"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -769,39 +541,39 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>controls</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>subcategory_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>_class</t>
+          <t>subcategory_examples</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>subcategory_status</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>props</t>
+          <t>subcategory_moved_to</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>parts</t>
+          <t>subcategory_incorporated_into</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"function,category,subcategory"</formula1>
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"withdrawn"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -809,175 +581,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>controls</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>_class</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>props</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>parts</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"function,category,subcategory"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>_class</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>props</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>parts</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"function,category,subcategory"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ns</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>prose</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ns</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>remarks</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -989,12 +592,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rel</t>
+          <t>implementation_example_id</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(schema): prefix the identifier keys with csf_
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/nist_csf_v2.xlsx
+++ b/project/excel/nist_csf_v2.xlsx
@@ -428,7 +428,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>functions</t>
+          <t>csf_functions</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>function_id</t>
+          <t>csf_function_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>category_id</t>
+          <t>csf_category_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>subcategory_id</t>
+          <t>csf_subcategory_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>implementation_example_id</t>
+          <t>csf_implementation_example_id</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(schema): key each inlined list by its identifier, not its title
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/nist_csf_v2.xlsx
+++ b/project/excel/nist_csf_v2.xlsx
@@ -449,17 +449,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>csf_function_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>csf_function_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -485,17 +485,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>csf_category_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>csf_category_id</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -541,12 +541,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>csf_subcategory_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>csf_subcategory_id</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -592,12 +592,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>csf_implementation_example_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>csf_implementation_example_id</t>
         </is>
       </c>
     </row>

</xml_diff>